<commit_message>
feat: ajustes mensagem de exibicao
</commit_message>
<xml_diff>
--- a/lista_usuarios.xlsx
+++ b/lista_usuarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\carometro_static\carometro-sesi-ce407\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B48D8C-6FBD-47D5-BE3C-35A145CDB449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF360B6F-1300-4661-A657-A4F42E595864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{56777C0C-48DE-4E81-9A5D-75EDE5A813EC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="115">
   <si>
     <t>funcao</t>
   </si>
@@ -320,27 +320,15 @@
     <t>Orientadora Educacional</t>
   </si>
   <si>
-    <t>Coordenado Ensino Fundamental</t>
-  </si>
-  <si>
     <t>Secretária</t>
   </si>
   <si>
-    <t>Coordenado Ensino Médio</t>
-  </si>
-  <si>
     <t>Bibliotecário</t>
   </si>
   <si>
     <t>Manutenção</t>
   </si>
   <si>
-    <t>Orientador de Educação Digital</t>
-  </si>
-  <si>
-    <t>Atualizar...</t>
-  </si>
-  <si>
     <t>visualizador</t>
   </si>
   <si>
@@ -375,13 +363,34 @@
   </si>
   <si>
     <t>718874</t>
+  </si>
+  <si>
+    <t>Cozinheira</t>
+  </si>
+  <si>
+    <t>Professora Tutora</t>
+  </si>
+  <si>
+    <t>Auxiliar de Cozinha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orientador de Educação Digital </t>
+  </si>
+  <si>
+    <t>Professora Educaçação Inclusiva</t>
+  </si>
+  <si>
+    <t>Coordenadora EF</t>
+  </si>
+  <si>
+    <t>Coordenadora EM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -391,6 +400,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -416,9 +432,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,7 +775,7 @@
   <cols>
     <col min="1" max="1" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -777,12 +794,12 @@
         <v>83</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>39</v>
@@ -791,10 +808,10 @@
         <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -808,10 +825,10 @@
         <v>87</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -825,10 +842,10 @@
         <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -839,13 +856,13 @@
         <v>42</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -859,10 +876,10 @@
         <v>88</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -873,13 +890,13 @@
         <v>44</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -890,13 +907,13 @@
         <v>45</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E8" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -910,10 +927,10 @@
         <v>87</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -927,10 +944,10 @@
         <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -944,10 +961,10 @@
         <v>87</v>
       </c>
       <c r="D11" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E11" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -961,10 +978,10 @@
         <v>87</v>
       </c>
       <c r="D12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -978,10 +995,10 @@
         <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -992,13 +1009,13 @@
         <v>51</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1009,13 +1026,13 @@
         <v>52</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E15" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -1029,32 +1046,32 @@
         <v>89</v>
       </c>
       <c r="D16" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E16" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E17" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>54</v>
@@ -1063,15 +1080,15 @@
         <v>87</v>
       </c>
       <c r="D18" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>55</v>
@@ -1080,10 +1097,10 @@
         <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1097,10 +1114,10 @@
         <v>87</v>
       </c>
       <c r="D20" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -1114,10 +1131,10 @@
         <v>87</v>
       </c>
       <c r="D21" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E21" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1131,10 +1148,10 @@
         <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E22" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1148,10 +1165,10 @@
         <v>91</v>
       </c>
       <c r="D23" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1162,18 +1179,18 @@
         <v>60</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D24" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E24" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>61</v>
@@ -1182,10 +1199,10 @@
         <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E25" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -1199,15 +1216,15 @@
         <v>92</v>
       </c>
       <c r="D26" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E26" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>63</v>
@@ -1216,10 +1233,10 @@
         <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E27" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -1233,10 +1250,10 @@
         <v>87</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -1247,13 +1264,13 @@
         <v>65</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1267,27 +1284,27 @@
         <v>90</v>
       </c>
       <c r="D30" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E30" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D31" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E31" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -1298,13 +1315,13 @@
         <v>68</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D32" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E32" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1315,13 +1332,13 @@
         <v>69</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D33" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E33" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1335,10 +1352,10 @@
         <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E34" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1352,10 +1369,10 @@
         <v>88</v>
       </c>
       <c r="D35" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E35" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -1369,10 +1386,10 @@
         <v>90</v>
       </c>
       <c r="D36" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E36" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -1386,10 +1403,10 @@
         <v>90</v>
       </c>
       <c r="D37" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E37" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -1403,10 +1420,10 @@
         <v>91</v>
       </c>
       <c r="D38" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E38" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -1417,13 +1434,13 @@
         <v>75</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="D39" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E39" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1433,14 +1450,14 @@
       <c r="B40" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>99</v>
+      <c r="C40" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="D40" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E40" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -1451,13 +1468,13 @@
         <v>77</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E41" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -1468,13 +1485,13 @@
         <v>78</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D42" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E42" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1488,10 +1505,10 @@
         <v>87</v>
       </c>
       <c r="D43" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E43" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1505,10 +1522,10 @@
         <v>88</v>
       </c>
       <c r="D44" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E44" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -1522,10 +1539,10 @@
         <v>87</v>
       </c>
       <c r="D45" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E45" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -1539,10 +1556,10 @@
         <v>88</v>
       </c>
       <c r="D46" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E46" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>